<commit_message>
Fix UK/USA country casing; make cleaning script reproducible from repo
</commit_message>
<xml_diff>
--- a/metadata/ECRMDP_Business_Glossary.xlsx
+++ b/metadata/ECRMDP_Business_Glossary.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="464">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="465">
   <si>
     <t xml:space="preserve">ECRMDP - CRM Business Glossary (UC16, Sprint 3)</t>
   </si>
@@ -42,7 +42,7 @@
     <t xml:space="preserve">Built from</t>
   </si>
   <si>
-    <t xml:space="preserve">The actual data in datasets/*_silver.csv and the warehouse schema (sql/Silver.sql), checked at repo commit 3001bf2; stakeholders from docs/BRD Document.docx.</t>
+    <t xml:space="preserve">The actual data in datasets/*_silver.csv and the warehouse schema (sql/Silver.sql), checked at repo commit 4a12a46; stakeholders from docs/BRD Document.docx.</t>
   </si>
   <si>
     <t xml:space="preserve">Business owners</t>
@@ -171,7 +171,7 @@
     <t xml:space="preserve">Age in years; income in source currency (currency not stated in source)</t>
   </si>
   <si>
-    <t xml:space="preserve">Age 18-69; income 25,093-249,991; gender Female/Male/Other; education Graduate/High School/PhD/Postgraduate; marital status Divorced/Married/Single</t>
+    <t xml:space="preserve">Age 18-69; income 25,093-249,991; gender Female/Male/Other; education Graduate/High School/PhD/Postgraduate; marital status Divorced/Married/Single; country Australia/France/Germany/India/Singapore/UK/USA</t>
   </si>
   <si>
     <t xml:space="preserve">Registration date</t>
@@ -1326,25 +1326,28 @@
     <t xml:space="preserve">silver/cleansing/data_cleaning.py line 52</t>
   </si>
   <si>
+    <t xml:space="preserve">Fixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Script now restores UK/USA after Title Case; customer_master_silver.csv regenerated (559 rows corrected: 296 UK, 263 USA).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DQ2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data dictionary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/CRM_Data_Dictionary lists fields that are not in the delivered data (e.g. phone, date_of_birth, assigned_to, expected_value, opportunity_name).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Readers of the dictionary will look for columns that do not exist.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/CRM_Data_Dictionary (1).xlsx</t>
+  </si>
+  <si>
     <t xml:space="preserve">Open</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stop title-casing acronyms (e.g. map 'Uk'-&gt;'UK', 'Usa'-&gt;'USA') and regenerate silver; or fix in Power Query.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DQ2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data dictionary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/CRM_Data_Dictionary lists fields that are not in the delivered data (e.g. phone, date_of_birth, assigned_to, expected_value, opportunity_name).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Readers of the dictionary will look for columns that do not exist.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">docs/CRM_Data_Dictionary (1).xlsx</t>
   </si>
   <si>
     <t xml:space="preserve">Align the dictionary with the actual source columns (see metadata/ECRMDP_Source_to_Target_Mapping.xlsx, Bronze_Mapping).</t>
@@ -2169,7 +2172,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
         <v>44</v>
       </c>
@@ -4493,7 +4496,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
         <v>427</v>
       </c>
@@ -4533,102 +4536,102 @@
         <v>438</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>197</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>207</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
     </row>
   </sheetData>

</xml_diff>